<commit_message>
Updates CCS economic deployment code, reads parameters from input data, updates to data (in-progress #11)
</commit_message>
<xml_diff>
--- a/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
+++ b/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\ccs\BCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\ccs\BCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F268FE25-6FA1-4964-97BE-7705BD55074C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC5397E-7CBE-4A89-A625-51FDEE7B98C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="58815" yWindow="1155" windowWidth="22695" windowHeight="14475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="Electricity Calculations" sheetId="5" r:id="rId2"/>
-    <sheet name="BCS-BCS" sheetId="4" r:id="rId3"/>
-    <sheet name="BCS-DoSfCS" sheetId="6" r:id="rId4"/>
+    <sheet name="45Q Value" sheetId="7" r:id="rId2"/>
+    <sheet name="Electricity Calculations" sheetId="5" r:id="rId3"/>
+    <sheet name="BCS-BCS" sheetId="4" r:id="rId4"/>
+    <sheet name="BCS-DoSfCS" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">About!$A$11</definedName>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
   <si>
     <t>Source:</t>
   </si>
@@ -119,16 +120,108 @@
   </si>
   <si>
     <t>12 years</t>
+  </si>
+  <si>
+    <t>Historical Consumer Price Index for All Urban Consumers (CPI-U): U.S. city average, all items, index</t>
+  </si>
+  <si>
+    <t>averages — Continued</t>
+  </si>
+  <si>
+    <t>[1982-84=100, unless otherwise noted]</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Annual avg.</t>
+  </si>
+  <si>
+    <t>Percent change from previous</t>
+  </si>
+  <si>
+    <t>Multiply by to get 2012 Dollars</t>
+  </si>
+  <si>
+    <t>Dec.</t>
+  </si>
+  <si>
+    <t>2012............................................................................. .</t>
+  </si>
+  <si>
+    <t>2013............................................................................. .</t>
+  </si>
+  <si>
+    <t>2014............................................................................. .</t>
+  </si>
+  <si>
+    <t>2015............................................................................. .</t>
+  </si>
+  <si>
+    <t>2016............................................................................. .</t>
+  </si>
+  <si>
+    <t>2017............................................................................. .</t>
+  </si>
+  <si>
+    <t>2018............................................................................. .</t>
+  </si>
+  <si>
+    <t>2019............................................................................. .</t>
+  </si>
+  <si>
+    <t>2020............................................................................. .</t>
+  </si>
+  <si>
+    <t>2021............................................................................. .</t>
+  </si>
+  <si>
+    <t>2022............................................................................. .</t>
+  </si>
+  <si>
+    <t>2023............................................................................. .</t>
+  </si>
+  <si>
+    <t>2024............................................................................. .</t>
+  </si>
+  <si>
+    <t>For geologically stored CO2</t>
+  </si>
+  <si>
+    <t>equipment placed in service 2/8/18 to 1/1/23</t>
+  </si>
+  <si>
+    <t>https://www.congress.gov/crs-product/IF11455</t>
+  </si>
+  <si>
+    <t>equipment placed in service 1/1/23-1/1/33</t>
+  </si>
+  <si>
+    <t>Future inflation assumption</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>2025…</t>
+  </si>
+  <si>
+    <t>2026…</t>
+  </si>
+  <si>
+    <t>2027…</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="#0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,6 +243,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -174,17 +273,21 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -491,20 +594,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F37"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" customWidth="1"/>
-    <col min="2" max="2" width="55.88671875" customWidth="1"/>
-    <col min="4" max="4" width="30.5546875" customWidth="1"/>
+    <col min="1" max="1" width="30.36328125" customWidth="1"/>
+    <col min="2" max="2" width="55.90625" customWidth="1"/>
+    <col min="4" max="4" width="30.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,43 +615,343 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="5">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
         <v>0.78500000000000003</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="5">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>17</v>
       </c>
       <c r="B13" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="8">
+        <v>229.59399999999999</v>
+      </c>
+      <c r="C20">
+        <v>1.7</v>
+      </c>
+      <c r="D20">
+        <v>2.1</v>
+      </c>
+      <c r="E20" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="8">
+        <v>232.95699999999999</v>
+      </c>
+      <c r="C21">
+        <v>1.5</v>
+      </c>
+      <c r="D21">
+        <v>1.5</v>
+      </c>
+      <c r="E21" s="7">
+        <v>0.98556385942470071</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="8">
+        <v>236.73599999999999</v>
+      </c>
+      <c r="C22">
+        <v>0.8</v>
+      </c>
+      <c r="D22">
+        <v>1.6</v>
+      </c>
+      <c r="E22" s="7">
+        <v>0.96983137334414704</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="8">
+        <v>237.017</v>
+      </c>
+      <c r="C23">
+        <v>0.7</v>
+      </c>
+      <c r="D23">
+        <v>0.1</v>
+      </c>
+      <c r="E23" s="7">
+        <v>0.9686815713640794</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="8">
+        <v>240.00700000000001</v>
+      </c>
+      <c r="C24">
+        <v>2.1</v>
+      </c>
+      <c r="D24">
+        <v>1.3</v>
+      </c>
+      <c r="E24" s="7">
+        <v>0.95661376543184151</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="8">
+        <v>245.12</v>
+      </c>
+      <c r="C25">
+        <v>2.1</v>
+      </c>
+      <c r="D25">
+        <v>2.1</v>
+      </c>
+      <c r="E25" s="7">
+        <v>0.93665959530026111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="8">
+        <v>251.107</v>
+      </c>
+      <c r="C26">
+        <v>1.9</v>
+      </c>
+      <c r="D26">
+        <v>2.4</v>
+      </c>
+      <c r="E26" s="7">
+        <v>0.9143273584567535</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="8">
+        <v>255.65700000000001</v>
+      </c>
+      <c r="C27">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D27">
+        <v>1.8</v>
+      </c>
+      <c r="E27" s="7">
+        <v>0.89805481563188172</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="8">
+        <v>258.81099999999998</v>
+      </c>
+      <c r="C28">
+        <v>1.4</v>
+      </c>
+      <c r="D28">
+        <v>1.2</v>
+      </c>
+      <c r="E28" s="7">
+        <v>0.88711067149387013</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="8">
+        <v>270.97000000000003</v>
+      </c>
+      <c r="C29">
+        <v>7</v>
+      </c>
+      <c r="D29">
+        <v>4.7</v>
+      </c>
+      <c r="E29" s="7">
+        <v>0.84730412960844359</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" s="8">
+        <v>292.65499999999997</v>
+      </c>
+      <c r="C30">
+        <v>6.5</v>
+      </c>
+      <c r="D30">
+        <v>8</v>
+      </c>
+      <c r="E30" s="7">
+        <v>0.78452102304761584</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="8">
+        <v>304.702</v>
+      </c>
+      <c r="E31" s="7">
+        <v>0.75350342301658668</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32">
+        <v>313.68900000000002</v>
+      </c>
+      <c r="E32" s="7">
+        <v>0.73191600598044548</v>
+      </c>
+      <c r="F32">
+        <f>B20/B32</f>
+        <v>0.73191600598044548</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="7">
+        <f>B32/(1-$B$37/100)</f>
+        <v>321.7323076923077</v>
+      </c>
+      <c r="E33" s="7">
+        <f>$B$20/B33</f>
+        <v>0.71361810583093443</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="7">
+        <f>B33/(1-$B$37/100)</f>
+        <v>329.9818540433925</v>
+      </c>
+      <c r="E34" s="7">
+        <f>$B$20/B34</f>
+        <v>0.69577765318516105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="7">
+        <f>B34/(1-$B$37/100)</f>
+        <v>338.44292722399234</v>
+      </c>
+      <c r="E35" s="7">
+        <f>$B$20/B35</f>
+        <v>0.67838321185553196</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37">
+        <v>2.5</v>
+      </c>
+      <c r="C37" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -558,45 +961,127 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AB35C55-7F27-44A6-A8A7-496D78F28576}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF232AA2-07A6-4879-829D-45E06644D581}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="38.08984375" customWidth="1"/>
+    <col min="3" max="3" width="37.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="7">
-        <f>About!B11</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="C7">
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="7">
-        <f>B1*B3/B2</f>
-        <v>51</v>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="C8">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="C9">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>2026</v>
+      </c>
+      <c r="C10">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>2027</v>
+      </c>
+      <c r="C11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>2028</v>
+      </c>
+      <c r="C12">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>2029</v>
+      </c>
+      <c r="C13">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>2030</v>
+      </c>
+      <c r="C14">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>2031</v>
+      </c>
+      <c r="C15">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>2032</v>
+      </c>
+      <c r="C16">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -605,320 +1090,45 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <sheetPr>
-    <tabColor theme="3"/>
-  </sheetPr>
-  <dimension ref="A1:AE3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AB35C55-7F27-44A6-A8A7-496D78F28576}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="24.5546875" customWidth="1"/>
+    <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="2">
-        <v>2021</v>
-      </c>
-      <c r="C1" s="2">
-        <v>2022</v>
-      </c>
-      <c r="D1" s="2">
-        <v>2023</v>
-      </c>
-      <c r="E1" s="2">
-        <v>2024</v>
-      </c>
-      <c r="F1" s="2">
-        <v>2025</v>
-      </c>
-      <c r="G1" s="2">
-        <v>2026</v>
-      </c>
-      <c r="H1" s="2">
-        <v>2027</v>
-      </c>
-      <c r="I1" s="2">
-        <v>2028</v>
-      </c>
-      <c r="J1" s="2">
-        <v>2029</v>
-      </c>
-      <c r="K1" s="2">
-        <v>2030</v>
-      </c>
-      <c r="L1" s="2">
-        <v>2031</v>
-      </c>
-      <c r="M1" s="2">
-        <v>2032</v>
-      </c>
-      <c r="N1" s="2">
-        <v>2033</v>
-      </c>
-      <c r="O1" s="2">
-        <v>2034</v>
-      </c>
-      <c r="P1" s="2">
-        <v>2035</v>
-      </c>
-      <c r="Q1" s="2">
-        <v>2036</v>
-      </c>
-      <c r="R1" s="2">
-        <v>2037</v>
-      </c>
-      <c r="S1" s="2">
-        <v>2038</v>
-      </c>
-      <c r="T1" s="2">
-        <v>2039</v>
-      </c>
-      <c r="U1" s="2">
-        <v>2040</v>
-      </c>
-      <c r="V1" s="2">
-        <v>2041</v>
-      </c>
-      <c r="W1" s="2">
-        <v>2042</v>
-      </c>
-      <c r="X1" s="2">
-        <v>2043</v>
-      </c>
-      <c r="Y1" s="2">
-        <v>2044</v>
-      </c>
-      <c r="Z1" s="2">
-        <v>2045</v>
-      </c>
-      <c r="AA1" s="2">
-        <v>2046</v>
-      </c>
-      <c r="AB1" s="2">
-        <v>2047</v>
-      </c>
-      <c r="AC1" s="2">
-        <v>2048</v>
-      </c>
-      <c r="AD1" s="2">
-        <v>2049</v>
-      </c>
-      <c r="AE1" s="2">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="B1" s="6">
+        <f>About!B11</f>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="4">
-        <v>0</v>
-      </c>
-      <c r="C2" s="4">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="E2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="F2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="G2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="H2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="I2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="J2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="K2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="L2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="M2">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
-      </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-      <c r="X2">
-        <v>0</v>
-      </c>
-      <c r="Y2">
-        <v>0</v>
-      </c>
-      <c r="Z2">
-        <v>0</v>
-      </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-      <c r="AC2">
-        <v>0</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="4">
-        <v>0</v>
-      </c>
-      <c r="C3" s="4">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="E3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="F3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="G3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="H3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="I3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="J3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="K3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="L3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="M3">
-        <f>About!$B$11*About!$A$9</f>
-        <v>66.725000000000009</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3">
-        <v>0</v>
-      </c>
-      <c r="U3">
-        <v>0</v>
-      </c>
-      <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <v>0</v>
-      </c>
-      <c r="X3">
-        <v>0</v>
-      </c>
-      <c r="Y3">
-        <v>0</v>
-      </c>
-      <c r="Z3">
-        <v>0</v>
-      </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AB3">
-        <v>0</v>
-      </c>
-      <c r="AC3">
-        <v>0</v>
-      </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
-      <c r="AE3">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="6">
+        <f>B1*B3/B2</f>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -927,14 +1137,358 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
+    <tabColor theme="3"/>
+  </sheetPr>
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.453125" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="2">
+        <v>2023</v>
+      </c>
+      <c r="E1" s="2">
+        <v>2024</v>
+      </c>
+      <c r="F1" s="2">
+        <v>2025</v>
+      </c>
+      <c r="G1" s="2">
+        <v>2026</v>
+      </c>
+      <c r="H1" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I1" s="2">
+        <v>2028</v>
+      </c>
+      <c r="J1" s="2">
+        <v>2029</v>
+      </c>
+      <c r="K1" s="2">
+        <v>2030</v>
+      </c>
+      <c r="L1" s="2">
+        <v>2031</v>
+      </c>
+      <c r="M1" s="2">
+        <v>2032</v>
+      </c>
+      <c r="N1" s="2">
+        <v>2033</v>
+      </c>
+      <c r="O1" s="2">
+        <v>2034</v>
+      </c>
+      <c r="P1" s="2">
+        <v>2035</v>
+      </c>
+      <c r="Q1" s="2">
+        <v>2036</v>
+      </c>
+      <c r="R1" s="2">
+        <v>2037</v>
+      </c>
+      <c r="S1" s="2">
+        <v>2038</v>
+      </c>
+      <c r="T1" s="2">
+        <v>2039</v>
+      </c>
+      <c r="U1" s="2">
+        <v>2040</v>
+      </c>
+      <c r="V1" s="2">
+        <v>2041</v>
+      </c>
+      <c r="W1" s="2">
+        <v>2042</v>
+      </c>
+      <c r="X1" s="2">
+        <v>2043</v>
+      </c>
+      <c r="Y1" s="2">
+        <v>2044</v>
+      </c>
+      <c r="Z1" s="2">
+        <v>2045</v>
+      </c>
+      <c r="AA1" s="2">
+        <v>2046</v>
+      </c>
+      <c r="AB1" s="2">
+        <v>2047</v>
+      </c>
+      <c r="AC1" s="2">
+        <v>2048</v>
+      </c>
+      <c r="AD1" s="2">
+        <v>2049</v>
+      </c>
+      <c r="AE1" s="2">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="9">
+        <f>'45Q Value'!B5*About!E29</f>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C2" s="9">
+        <f>'45Q Value'!B6*About!E30</f>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D2" s="9">
+        <f>'45Q Value'!C7*About!E31</f>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E2" s="9">
+        <f>'45Q Value'!C8*About!E32</f>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F2" s="9">
+        <f>'45Q Value'!C9*About!E33</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G2" s="9">
+        <f>'45Q Value'!C10*About!E34</f>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H2" s="9">
+        <f>$F$2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I2" s="9">
+        <f t="shared" ref="I2:M2" si="0">H2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J2" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K2" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L2" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M2" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="9">
+        <f t="shared" ref="B3:C3" si="1">B2</f>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C3" s="9">
+        <f t="shared" si="1"/>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D3" s="9">
+        <f>D2</f>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E3" s="9">
+        <f t="shared" ref="E3:AE3" si="2">E2</f>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F3" s="9">
+        <f t="shared" si="2"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G3" s="9">
+        <f t="shared" si="2"/>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H3" s="9">
+        <f t="shared" si="2"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I3" s="9">
+        <f t="shared" si="2"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J3" s="9">
+        <f t="shared" si="2"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K3" s="9">
+        <f t="shared" si="2"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L3" s="9">
+        <f t="shared" si="2"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M3" s="9">
+        <f t="shared" si="2"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5698252-CD29-4D86-9D7F-2214C5598602}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1029,7 +1583,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Integrate 4.0.4: commit #c9cf68b, 3/25/25, Update BAU industry CCS subsidies for tax credit duration (*extend indst timeline not power*)
</commit_message>
<xml_diff>
--- a/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
+++ b/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
@@ -1,24 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\ccs\BCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\ccs\BCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC5397E-7CBE-4A89-A625-51FDEE7B98C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC7E4D8-CE5D-4DA0-BF00-EE6F226ECBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58815" yWindow="1155" windowWidth="22695" windowHeight="14475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="45Q Value" sheetId="7" r:id="rId2"/>
     <sheet name="Electricity Calculations" sheetId="5" r:id="rId3"/>
-    <sheet name="BCS-BCS" sheetId="4" r:id="rId4"/>
-    <sheet name="BCS-DoSfCS" sheetId="6" r:id="rId5"/>
+    <sheet name="Calculations" sheetId="8" r:id="rId4"/>
+    <sheet name="BCS-BCS" sheetId="4" r:id="rId5"/>
+    <sheet name="BCS-DoSfCS" sheetId="6" r:id="rId6"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId7"/>
+  </externalReferences>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">About!$A$11</definedName>
     <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
@@ -63,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="88">
   <si>
     <t>Source:</t>
   </si>
@@ -210,6 +214,123 @@
   </si>
   <si>
     <t>2027…</t>
+  </si>
+  <si>
+    <t>45Q phase-in period</t>
+  </si>
+  <si>
+    <t>45Q phase-out period</t>
+  </si>
+  <si>
+    <t>*We use the data below for calculating the fraction of CCS potential achieved by industry. We do not subscript 45Q tax credits by sub-industry, so we must</t>
+  </si>
+  <si>
+    <t>choose a representative value for determining how to apply a duration multiplier. Since most of the incremental CCS comes online between 2030-2035, we use that timeline.</t>
+  </si>
+  <si>
+    <t>The potentials below use the "High emissions" values from the Rhodium figure above and are presented as MMT of capture capacity.</t>
+  </si>
+  <si>
+    <t>agriculture and forestry 01T03</t>
+  </si>
+  <si>
+    <t>coal mining 05</t>
+  </si>
+  <si>
+    <t>oil and gas extraction 06</t>
+  </si>
+  <si>
+    <t>other mining and quarrying 07T08</t>
+  </si>
+  <si>
+    <t>food beverage and tobacco 10T12</t>
+  </si>
+  <si>
+    <t>textiles apparel and leather 13T15</t>
+  </si>
+  <si>
+    <t>wood products 16</t>
+  </si>
+  <si>
+    <t>pulp paper and printing 17T18</t>
+  </si>
+  <si>
+    <t>refined petroleum and coke 19 - energy</t>
+  </si>
+  <si>
+    <t>*mapped to energy-related emissions rather than process emissions, since CCS equipment is installed on crackers</t>
+  </si>
+  <si>
+    <t>refined petroleum and coke 19 - process</t>
+  </si>
+  <si>
+    <t>*mapped to process emissions</t>
+  </si>
+  <si>
+    <t>chemicals 20</t>
+  </si>
+  <si>
+    <t>*ammonia not counted because we assume this industry is decarbonized through the hydrogen PTC</t>
+  </si>
+  <si>
+    <t>rubber and plastic products 22</t>
+  </si>
+  <si>
+    <t>glass and glass products 231</t>
+  </si>
+  <si>
+    <t>cement and other nonmetallic minerals 239</t>
+  </si>
+  <si>
+    <t>iron and steel 241</t>
+  </si>
+  <si>
+    <t>other metals 242</t>
+  </si>
+  <si>
+    <t>metal products except machinery and vehicles 25</t>
+  </si>
+  <si>
+    <t>computers and electronics 26</t>
+  </si>
+  <si>
+    <t>appliances and electrical equipment 27</t>
+  </si>
+  <si>
+    <t>other machinery 28</t>
+  </si>
+  <si>
+    <t>road vehicles 29</t>
+  </si>
+  <si>
+    <t>nonroad vehicles 30</t>
+  </si>
+  <si>
+    <t>other manufacturing 31T33</t>
+  </si>
+  <si>
+    <t>energy pipelines and gas processing 352T353</t>
+  </si>
+  <si>
+    <t>water and waste 36T39</t>
+  </si>
+  <si>
+    <t>construction 41T43</t>
+  </si>
+  <si>
+    <t>45Q tax credits include a commenced construction provision. Based on EIA data, we assume a construction timeline</t>
+  </si>
+  <si>
+    <t>of 3 years for the electricity sector.</t>
+  </si>
+  <si>
+    <t>The electricity sector calculations properly apply the tax credit duration depending on when CCS capacity comes online.</t>
+  </si>
+  <si>
+    <t>However, the industry sector does not have stock tracking for CCS equipment. Therefore, we adjust the BAU subsidy</t>
+  </si>
+  <si>
+    <t>values for industry only to reflect the duration multiplier.</t>
   </si>
 </sst>
 </file>
@@ -218,8 +339,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="#0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="#0.000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -273,7 +394,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -283,11 +404,14 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -305,6 +429,34 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="About"/>
+      <sheetName val="Calculations"/>
+      <sheetName val="BCS-BCS"/>
+      <sheetName val="BCS-DoSfCS"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3">
+        <row r="2">
+          <cell r="B2">
+            <v>12</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -594,20 +746,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F44"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.36328125" customWidth="1"/>
-    <col min="2" max="2" width="55.90625" customWidth="1"/>
-    <col min="4" max="4" width="30.54296875" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="2" max="2" width="55.85546875" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -615,22 +767,22 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>0.78500000000000003</v>
       </c>
@@ -638,7 +790,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -646,7 +798,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -654,22 +806,22 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -683,7 +835,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>26</v>
       </c>
@@ -691,7 +843,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -708,7 +860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -725,7 +877,7 @@
         <v>0.98556385942470071</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -742,7 +894,7 @@
         <v>0.96983137334414704</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -759,7 +911,7 @@
         <v>0.9686815713640794</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -776,7 +928,7 @@
         <v>0.95661376543184151</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -793,7 +945,7 @@
         <v>0.93665959530026111</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -810,7 +962,7 @@
         <v>0.9143273584567535</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -827,7 +979,7 @@
         <v>0.89805481563188172</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -844,7 +996,7 @@
         <v>0.88711067149387013</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -861,7 +1013,7 @@
         <v>0.84730412960844359</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -878,7 +1030,7 @@
         <v>0.78452102304761584</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -889,7 +1041,7 @@
         <v>0.75350342301658668</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>39</v>
       </c>
@@ -904,7 +1056,7 @@
         <v>0.73191600598044548</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>46</v>
       </c>
@@ -917,7 +1069,7 @@
         <v>0.71361810583093443</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>47</v>
       </c>
@@ -930,7 +1082,7 @@
         <v>0.69577765318516105</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>48</v>
       </c>
@@ -943,7 +1095,7 @@
         <v>0.67838321185553196</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>44</v>
       </c>
@@ -952,6 +1104,31 @@
       </c>
       <c r="C37" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -963,24 +1140,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF232AA2-07A6-4879-829D-45E06644D581}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="38.08984375" customWidth="1"/>
-    <col min="3" max="3" width="37.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.140625" customWidth="1"/>
+    <col min="3" max="3" width="37.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>41</v>
       </c>
@@ -988,7 +1165,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -996,7 +1173,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1004,7 +1181,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1012,7 +1189,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -1020,7 +1197,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2025</v>
       </c>
@@ -1028,7 +1205,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -1036,7 +1213,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2027</v>
       </c>
@@ -1044,7 +1221,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2028</v>
       </c>
@@ -1052,7 +1229,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2029</v>
       </c>
@@ -1060,7 +1237,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2030</v>
       </c>
@@ -1068,7 +1245,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2031</v>
       </c>
@@ -1076,7 +1253,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2032</v>
       </c>
@@ -1092,12 +1269,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AB35C55-7F27-44A6-A8A7-496D78F28576}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -1106,7 +1283,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1114,7 +1291,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1122,7 +1299,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1137,342 +1314,538 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <sheetPr>
-    <tabColor theme="3"/>
-  </sheetPr>
-  <dimension ref="A1:AE3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751291F6-B2A0-44B5-ABEB-B83CAA025A34}">
+  <dimension ref="A1:AE34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.453125" customWidth="1"/>
-    <col min="2" max="2" width="24.54296875" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="2">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="B1" s="10">
         <v>2021</v>
       </c>
-      <c r="C1" s="2">
+      <c r="C1">
         <v>2022</v>
       </c>
-      <c r="D1" s="2">
+      <c r="D1" s="10">
         <v>2023</v>
       </c>
-      <c r="E1" s="2">
+      <c r="E1">
         <v>2024</v>
       </c>
-      <c r="F1" s="2">
+      <c r="F1" s="10">
         <v>2025</v>
       </c>
-      <c r="G1" s="2">
+      <c r="G1">
         <v>2026</v>
       </c>
-      <c r="H1" s="2">
+      <c r="H1" s="10">
         <v>2027</v>
       </c>
-      <c r="I1" s="2">
+      <c r="I1">
         <v>2028</v>
       </c>
-      <c r="J1" s="2">
+      <c r="J1" s="10">
         <v>2029</v>
       </c>
-      <c r="K1" s="2">
+      <c r="K1">
         <v>2030</v>
       </c>
-      <c r="L1" s="2">
+      <c r="L1" s="10">
         <v>2031</v>
       </c>
-      <c r="M1" s="2">
+      <c r="M1">
         <v>2032</v>
       </c>
-      <c r="N1" s="2">
+      <c r="N1" s="10">
         <v>2033</v>
       </c>
-      <c r="O1" s="2">
+      <c r="O1">
         <v>2034</v>
       </c>
-      <c r="P1" s="2">
+      <c r="P1" s="10">
         <v>2035</v>
       </c>
-      <c r="Q1" s="2">
+      <c r="Q1">
         <v>2036</v>
       </c>
-      <c r="R1" s="2">
+      <c r="R1" s="10">
         <v>2037</v>
       </c>
-      <c r="S1" s="2">
+      <c r="S1">
         <v>2038</v>
       </c>
-      <c r="T1" s="2">
+      <c r="T1" s="10">
         <v>2039</v>
       </c>
-      <c r="U1" s="2">
+      <c r="U1">
         <v>2040</v>
       </c>
-      <c r="V1" s="2">
+      <c r="V1" s="10">
         <v>2041</v>
       </c>
-      <c r="W1" s="2">
+      <c r="W1">
         <v>2042</v>
       </c>
-      <c r="X1" s="2">
+      <c r="X1" s="10">
         <v>2043</v>
       </c>
-      <c r="Y1" s="2">
+      <c r="Y1">
         <v>2044</v>
       </c>
-      <c r="Z1" s="2">
+      <c r="Z1" s="10">
         <v>2045</v>
       </c>
-      <c r="AA1" s="2">
+      <c r="AA1">
         <v>2046</v>
       </c>
-      <c r="AB1" s="2">
+      <c r="AB1" s="10">
         <v>2047</v>
       </c>
-      <c r="AC1" s="2">
+      <c r="AC1">
         <v>2048</v>
       </c>
-      <c r="AD1" s="2">
+      <c r="AD1" s="10">
         <v>2049</v>
       </c>
-      <c r="AE1" s="2">
+      <c r="AE1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <f>1/5</f>
+        <v>0.2</v>
+      </c>
+      <c r="M2">
+        <f>L2+1/5</f>
+        <v>0.4</v>
+      </c>
+      <c r="N2">
+        <f t="shared" ref="N2:P2" si="0">M2+1/5</f>
+        <v>0.60000000000000009</v>
+      </c>
+      <c r="O2">
+        <f t="shared" si="0"/>
+        <v>0.8</v>
+      </c>
+      <c r="P2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <f>IFERROR(IF(A3=1,1,INDEX($B$2:$AE$2,MATCH((B1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <f>IFERROR(IF(B3=1,1,INDEX($B$2:$AE$2,MATCH((C1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <f>IFERROR(IF(C3=1,1,INDEX($B$2:$AE$2,MATCH((D1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <f>IFERROR(IF(D3=1,1,INDEX($B$2:$AE$2,MATCH((E1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <f>IFERROR(IF(E3=1,1,INDEX($B$2:$AE$2,MATCH((F1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <f>IFERROR(IF(F3=1,1,INDEX($B$2:$AE$2,MATCH((G1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <f>IFERROR(IF(G3=1,1,INDEX($B$2:$AE$2,MATCH((H1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <f>IFERROR(IF(H3=1,1,INDEX($B$2:$AE$2,MATCH((I1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <f>IFERROR(IF(I3=1,1,INDEX($B$2:$AE$2,MATCH((J1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <f>IFERROR(IF(J3=1,1,INDEX($B$2:$AE$2,MATCH((K1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <f>IFERROR(IF(K3=1,1,INDEX($B$2:$AE$2,MATCH((L1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <f>IFERROR(IF(L3=1,1,INDEX($B$2:$AE$2,MATCH((M1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <f>IFERROR(IF(M3=1,1,INDEX($B$2:$AE$2,MATCH((N1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <f>IFERROR(IF(N3=1,1,INDEX($B$2:$AE$2,MATCH((O1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <f>IFERROR(IF(O3=1,1,INDEX($B$2:$AE$2,MATCH((P1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <f>IFERROR(IF(P3=1,1,INDEX($B$2:$AE$2,MATCH((Q1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <f>IFERROR(IF(Q3=1,1,INDEX($B$2:$AE$2,MATCH((R1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <f>IFERROR(IF(R3=1,1,INDEX($B$2:$AE$2,MATCH((S1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <f>IFERROR(IF(S3=1,1,INDEX($B$2:$AE$2,MATCH((T1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <f>IFERROR(IF(T3=1,1,INDEX($B$2:$AE$2,MATCH((U1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <f>IFERROR(IF(U3=1,1,INDEX($B$2:$AE$2,MATCH((V1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <f>IFERROR(IF(V3=1,1,INDEX($B$2:$AE$2,MATCH((W1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <f>IFERROR(IF(W3=1,1,INDEX($B$2:$AE$2,MATCH((X1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0.2</v>
+      </c>
+      <c r="Y3">
+        <f>IFERROR(IF(X3=1,1,INDEX($B$2:$AE$2,MATCH((Y1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0.4</v>
+      </c>
+      <c r="Z3">
+        <f>IFERROR(IF(Y3=1,1,INDEX($B$2:$AE$2,MATCH((Z1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0.60000000000000009</v>
+      </c>
+      <c r="AA3">
+        <f>IFERROR(IF(Z3=1,1,INDEX($B$2:$AE$2,MATCH((AA1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>0.8</v>
+      </c>
+      <c r="AB3">
+        <f>IFERROR(IF(AA3=1,1,INDEX($B$2:$AE$2,MATCH((AB1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>1</v>
+      </c>
+      <c r="AC3">
+        <f>IFERROR(IF(AB3=1,1,INDEX($B$2:$AE$2,MATCH((AC1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>1</v>
+      </c>
+      <c r="AD3">
+        <f>IFERROR(IF(AC3=1,1,INDEX($B$2:$AE$2,MATCH((AD1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>1</v>
+      </c>
+      <c r="AE3">
+        <f>IFERROR(IF(AD3=1,1,INDEX($B$2:$AE$2,MATCH((AE1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>2022</v>
+      </c>
+      <c r="C8">
+        <v>2030</v>
+      </c>
+      <c r="D8">
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11">
+        <v>14</v>
+      </c>
+      <c r="C11">
+        <v>16</v>
+      </c>
+      <c r="D11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>60</v>
+      </c>
+      <c r="E17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18">
         <v>2</v>
       </c>
-      <c r="B2" s="9">
-        <f>'45Q Value'!B5*About!E29</f>
-        <v>42.365206480422181</v>
-      </c>
-      <c r="C2" s="9">
-        <f>'45Q Value'!B6*About!E30</f>
-        <v>39.226051152380791</v>
-      </c>
-      <c r="D2" s="9">
-        <f>'45Q Value'!C7*About!E31</f>
-        <v>64.04779095640987</v>
-      </c>
-      <c r="E2" s="9">
-        <f>'45Q Value'!C8*About!E32</f>
-        <v>62.212860508337869</v>
-      </c>
-      <c r="F2" s="9">
-        <f>'45Q Value'!C9*About!E33</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="G2" s="9">
-        <f>'45Q Value'!C10*About!E34</f>
-        <v>59.141100520738689</v>
-      </c>
-      <c r="H2" s="9">
-        <f>$F$2</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="I2" s="9">
-        <f t="shared" ref="I2:M2" si="0">H2</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="J2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="K2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="L2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="M2" s="9">
-        <f t="shared" si="0"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
-      </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-      <c r="X2">
-        <v>0</v>
-      </c>
-      <c r="Y2">
-        <v>0</v>
-      </c>
-      <c r="Z2">
-        <v>0</v>
-      </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-      <c r="AC2">
-        <v>0</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="9">
-        <f t="shared" ref="B3:C3" si="1">B2</f>
-        <v>42.365206480422181</v>
-      </c>
-      <c r="C3" s="9">
-        <f t="shared" si="1"/>
-        <v>39.226051152380791</v>
-      </c>
-      <c r="D3" s="9">
-        <f>D2</f>
-        <v>64.04779095640987</v>
-      </c>
-      <c r="E3" s="9">
-        <f t="shared" ref="E3:AE3" si="2">E2</f>
-        <v>62.212860508337869</v>
-      </c>
-      <c r="F3" s="9">
-        <f t="shared" si="2"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="G3" s="9">
-        <f t="shared" si="2"/>
-        <v>59.141100520738689</v>
-      </c>
-      <c r="H3" s="9">
-        <f t="shared" si="2"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="I3" s="9">
-        <f t="shared" si="2"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="J3" s="9">
-        <f t="shared" si="2"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="K3" s="9">
-        <f t="shared" si="2"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="L3" s="9">
-        <f t="shared" si="2"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="M3" s="9">
-        <f t="shared" si="2"/>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="N3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE3">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="C18">
+        <v>53</v>
+      </c>
+      <c r="D18">
+        <v>53</v>
+      </c>
+      <c r="E18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1481,14 +1854,358 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
+    <tabColor theme="3"/>
+  </sheetPr>
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="2">
+        <v>2023</v>
+      </c>
+      <c r="E1" s="2">
+        <v>2024</v>
+      </c>
+      <c r="F1" s="2">
+        <v>2025</v>
+      </c>
+      <c r="G1" s="2">
+        <v>2026</v>
+      </c>
+      <c r="H1" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I1" s="2">
+        <v>2028</v>
+      </c>
+      <c r="J1" s="2">
+        <v>2029</v>
+      </c>
+      <c r="K1" s="2">
+        <v>2030</v>
+      </c>
+      <c r="L1" s="2">
+        <v>2031</v>
+      </c>
+      <c r="M1" s="2">
+        <v>2032</v>
+      </c>
+      <c r="N1" s="2">
+        <v>2033</v>
+      </c>
+      <c r="O1" s="2">
+        <v>2034</v>
+      </c>
+      <c r="P1" s="2">
+        <v>2035</v>
+      </c>
+      <c r="Q1" s="2">
+        <v>2036</v>
+      </c>
+      <c r="R1" s="2">
+        <v>2037</v>
+      </c>
+      <c r="S1" s="2">
+        <v>2038</v>
+      </c>
+      <c r="T1" s="2">
+        <v>2039</v>
+      </c>
+      <c r="U1" s="2">
+        <v>2040</v>
+      </c>
+      <c r="V1" s="2">
+        <v>2041</v>
+      </c>
+      <c r="W1" s="2">
+        <v>2042</v>
+      </c>
+      <c r="X1" s="2">
+        <v>2043</v>
+      </c>
+      <c r="Y1" s="2">
+        <v>2044</v>
+      </c>
+      <c r="Z1" s="2">
+        <v>2045</v>
+      </c>
+      <c r="AA1" s="2">
+        <v>2046</v>
+      </c>
+      <c r="AB1" s="2">
+        <v>2047</v>
+      </c>
+      <c r="AC1" s="2">
+        <v>2048</v>
+      </c>
+      <c r="AD1" s="2">
+        <v>2049</v>
+      </c>
+      <c r="AE1" s="2">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="9">
+        <f>B3</f>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C2" s="9">
+        <f>C3</f>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D2" s="9">
+        <f>D3</f>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E2" s="9">
+        <f>E3</f>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F2" s="9">
+        <f>F3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G2" s="9">
+        <f>G3</f>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H2" s="9">
+        <f>H3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I2" s="9">
+        <f>I3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J2" s="9">
+        <f>J3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K2" s="9">
+        <f>K3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L2" s="9">
+        <f>L3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M2" s="9">
+        <f>M3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="9">
+        <f>'45Q Value'!B5*About!E29</f>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C3" s="9">
+        <f>'45Q Value'!B6*About!E30</f>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D3" s="9">
+        <f>'45Q Value'!C7*About!E31</f>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E3" s="9">
+        <f>'45Q Value'!C8*About!E32</f>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F3" s="9">
+        <f>'45Q Value'!C9*About!E33</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G3" s="9">
+        <f>'45Q Value'!C10*About!E34</f>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H3" s="9">
+        <f>$F$3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I3" s="9">
+        <f t="shared" ref="I3:M3" si="0">H3</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J3" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K3" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L3" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M3" s="9">
+        <f t="shared" si="0"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N3" s="9">
+        <f>$M3*(1-Calculations!N3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="O3" s="9">
+        <f>$M3*(1-Calculations!O3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="P3" s="9">
+        <f>$M3*(1-Calculations!P3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="Q3" s="9">
+        <f>$M3*(1-Calculations!Q3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="R3" s="9">
+        <f>$M3*(1-Calculations!R3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="S3" s="9">
+        <f>$M3*(1-Calculations!S3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="T3" s="9">
+        <f>$M3*(1-Calculations!T3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="U3" s="9">
+        <f>$M3*(1-Calculations!U3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="V3" s="9">
+        <f>$M3*(1-Calculations!V3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="W3" s="9">
+        <f>$M3*(1-Calculations!W3)</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="X3" s="9">
+        <f>$M3*(1-Calculations!X3)</f>
+        <v>48.526031196503546</v>
+      </c>
+      <c r="Y3" s="9">
+        <f>$M3*(1-Calculations!Y3)</f>
+        <v>36.394523397377654</v>
+      </c>
+      <c r="Z3" s="9">
+        <f>$M3*(1-Calculations!Z3)</f>
+        <v>24.263015598251766</v>
+      </c>
+      <c r="AA3" s="9">
+        <f>$M3*(1-Calculations!AA3)</f>
+        <v>12.131507799125883</v>
+      </c>
+      <c r="AB3" s="9">
+        <f>$M3*(1-Calculations!AB3)</f>
+        <v>0</v>
+      </c>
+      <c r="AC3" s="9">
+        <f>$M3*(1-Calculations!AC3)</f>
+        <v>0</v>
+      </c>
+      <c r="AD3" s="9">
+        <f>$M3*(1-Calculations!AD3)</f>
+        <v>0</v>
+      </c>
+      <c r="AE3" s="9">
+        <f>$M3*(1-Calculations!AE3)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5698252-CD29-4D86-9D7F-2214C5598602}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1583,7 +2300,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Subscripts electricity sector CCS credit so it can be customized by power plant type (#330)
</commit_message>
<xml_diff>
--- a/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
+++ b/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\ccs\BCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ccs\BCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC7E4D8-CE5D-4DA0-BF00-EE6F226ECBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9F6EC0-2F2F-4CCB-BD1C-F954EC71A52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23730" yWindow="2610" windowWidth="21825" windowHeight="13170" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="45Q Value" sheetId="7" r:id="rId2"/>
     <sheet name="Electricity Calculations" sheetId="5" r:id="rId3"/>
     <sheet name="Calculations" sheetId="8" r:id="rId4"/>
-    <sheet name="BCS-BCS" sheetId="4" r:id="rId5"/>
-    <sheet name="BCS-DoSfCS" sheetId="6" r:id="rId6"/>
+    <sheet name="BCS-industry" sheetId="4" r:id="rId5"/>
+    <sheet name="BCS-electricity" sheetId="9" r:id="rId6"/>
+    <sheet name="BCS-DoSfCS" sheetId="6" r:id="rId7"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">About!$A$11</definedName>
@@ -67,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="112">
   <si>
     <t>Source:</t>
   </si>
@@ -75,9 +76,6 @@
     <t>Notes:</t>
   </si>
   <si>
-    <t>electricity sector</t>
-  </si>
-  <si>
     <t>industry sector</t>
   </si>
   <si>
@@ -331,6 +329,81 @@
   </si>
   <si>
     <t>values for industry only to reflect the duration multiplier.</t>
+  </si>
+  <si>
+    <t>Unit: dimensionless (% of project cost)</t>
+  </si>
+  <si>
+    <t>hard coal</t>
+  </si>
+  <si>
+    <t>natural gas steam turbine</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle</t>
+  </si>
+  <si>
+    <t>nuclear</t>
+  </si>
+  <si>
+    <t>hydro</t>
+  </si>
+  <si>
+    <t>onshore wind</t>
+  </si>
+  <si>
+    <t>solar PV</t>
+  </si>
+  <si>
+    <t>solar thermal</t>
+  </si>
+  <si>
+    <t>biomass</t>
+  </si>
+  <si>
+    <t>geothermal</t>
+  </si>
+  <si>
+    <t>petroleum</t>
+  </si>
+  <si>
+    <t>natural gas peaker</t>
+  </si>
+  <si>
+    <t>lignite</t>
+  </si>
+  <si>
+    <t>offshore wind</t>
+  </si>
+  <si>
+    <t>crude oil</t>
+  </si>
+  <si>
+    <t>heavy or residual fuel oil</t>
+  </si>
+  <si>
+    <t>municipal solid waste</t>
+  </si>
+  <si>
+    <t>hard coal w CCS</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle w CCS</t>
+  </si>
+  <si>
+    <t>biomass w CCS</t>
+  </si>
+  <si>
+    <t>lignite w CCS</t>
+  </si>
+  <si>
+    <t>small modular reactor</t>
+  </si>
+  <si>
+    <t>hydrogen combustion turbine</t>
+  </si>
+  <si>
+    <t>hydrogen combined cycle</t>
   </si>
 </sst>
 </file>
@@ -342,7 +415,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="#0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -371,6 +444,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -394,7 +474,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -412,6 +492,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -756,7 +837,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -764,7 +845,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -774,12 +855,12 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -787,12 +868,12 @@
         <v>0.78500000000000003</v>
       </c>
       <c r="B9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="5">
         <v>85</v>
@@ -800,52 +881,52 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
         <v>17</v>
-      </c>
-      <c r="B13" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
         <v>22</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>23</v>
       </c>
-      <c r="C18" t="s">
+      <c r="E18" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B20" s="8">
         <v>229.59399999999999</v>
@@ -862,7 +943,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B21" s="8">
         <v>232.95699999999999</v>
@@ -879,7 +960,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B22" s="8">
         <v>236.73599999999999</v>
@@ -896,7 +977,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" s="8">
         <v>237.017</v>
@@ -913,7 +994,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B24" s="8">
         <v>240.00700000000001</v>
@@ -930,7 +1011,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25" s="8">
         <v>245.12</v>
@@ -947,7 +1028,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B26" s="8">
         <v>251.107</v>
@@ -964,7 +1045,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B27" s="8">
         <v>255.65700000000001</v>
@@ -981,7 +1062,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28" s="8">
         <v>258.81099999999998</v>
@@ -998,7 +1079,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B29" s="8">
         <v>270.97000000000003</v>
@@ -1015,7 +1096,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B30" s="8">
         <v>292.65499999999997</v>
@@ -1032,7 +1113,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B31" s="8">
         <v>304.702</v>
@@ -1043,7 +1124,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32">
         <v>313.68900000000002</v>
@@ -1058,7 +1139,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B33" s="7">
         <f>B32/(1-$B$37/100)</f>
@@ -1071,7 +1152,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B34" s="7">
         <f>B33/(1-$B$37/100)</f>
@@ -1084,7 +1165,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B35" s="7">
         <f>B34/(1-$B$37/100)</f>
@@ -1097,38 +1178,38 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B37">
         <v>2.5</v>
       </c>
       <c r="C37" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1149,20 +1230,20 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1276,7 +1357,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="6">
         <f>About!B11</f>
@@ -1285,7 +1366,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>20</v>
@@ -1293,7 +1374,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>12</v>
@@ -1301,7 +1382,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="6">
         <f>B1*B3/B2</f>
@@ -1415,7 +1496,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1515,7 +1596,7 @@
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3">
         <f>IFERROR(IF(A3=1,1,INDEX($B$2:$AE$2,MATCH((B1-'[1]BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
@@ -1640,17 +1721,17 @@
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
@@ -1666,17 +1747,17 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11">
         <v>14</v>
@@ -1690,32 +1771,32 @@
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1727,12 +1808,12 @@
         <v>60</v>
       </c>
       <c r="E17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -1744,30 +1825,30 @@
         <v>53</v>
       </c>
       <c r="E18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" t="s">
         <v>66</v>
-      </c>
-      <c r="E19" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1781,7 +1862,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -1795,57 +1876,57 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1858,7 +1939,7 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
@@ -1867,7 +1948,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="2">
         <v>2021</v>
@@ -1965,230 +2046,123 @@
         <v>2</v>
       </c>
       <c r="B2" s="9">
-        <f>B3</f>
-        <v>42.365206480422181</v>
-      </c>
-      <c r="C2" s="9">
-        <f>C3</f>
-        <v>39.226051152380791</v>
-      </c>
-      <c r="D2" s="9">
-        <f>D3</f>
-        <v>64.04779095640987</v>
-      </c>
-      <c r="E2" s="9">
-        <f>E3</f>
-        <v>62.212860508337869</v>
-      </c>
-      <c r="F2" s="9">
-        <f>F3</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="G2" s="9">
-        <f>G3</f>
-        <v>59.141100520738689</v>
-      </c>
-      <c r="H2" s="9">
-        <f>H3</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="I2" s="9">
-        <f>I3</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="J2" s="9">
-        <f>J3</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="K2" s="9">
-        <f>K3</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="L2" s="9">
-        <f>L3</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="M2" s="9">
-        <f>M3</f>
-        <v>60.65753899562943</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
-      </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-      <c r="X2">
-        <v>0</v>
-      </c>
-      <c r="Y2">
-        <v>0</v>
-      </c>
-      <c r="Z2">
-        <v>0</v>
-      </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-      <c r="AC2">
-        <v>0</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="9">
         <f>'45Q Value'!B5*About!E29</f>
         <v>42.365206480422181</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C2" s="9">
         <f>'45Q Value'!B6*About!E30</f>
         <v>39.226051152380791</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D2" s="9">
         <f>'45Q Value'!C7*About!E31</f>
         <v>64.04779095640987</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E2" s="9">
         <f>'45Q Value'!C8*About!E32</f>
         <v>62.212860508337869</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F2" s="9">
         <f>'45Q Value'!C9*About!E33</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G2" s="9">
         <f>'45Q Value'!C10*About!E34</f>
         <v>59.141100520738689</v>
       </c>
-      <c r="H3" s="9">
-        <f>$F$3</f>
+      <c r="H2" s="9">
+        <f>$F$2</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="I3" s="9">
-        <f t="shared" ref="I3:M3" si="0">H3</f>
+      <c r="I2" s="9">
+        <f t="shared" ref="I2:M2" si="0">H2</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J2" s="9">
         <f t="shared" si="0"/>
         <v>60.65753899562943</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K2" s="9">
         <f t="shared" si="0"/>
         <v>60.65753899562943</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L2" s="9">
         <f t="shared" si="0"/>
         <v>60.65753899562943</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M2" s="9">
         <f t="shared" si="0"/>
         <v>60.65753899562943</v>
       </c>
-      <c r="N3" s="9">
-        <f>$M3*(1-Calculations!N3)</f>
+      <c r="N2" s="9">
+        <f>$M2*(1-Calculations!N3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="O3" s="9">
-        <f>$M3*(1-Calculations!O3)</f>
+      <c r="O2" s="9">
+        <f>$M2*(1-Calculations!O3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="P3" s="9">
-        <f>$M3*(1-Calculations!P3)</f>
+      <c r="P2" s="9">
+        <f>$M2*(1-Calculations!P3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="Q3" s="9">
-        <f>$M3*(1-Calculations!Q3)</f>
+      <c r="Q2" s="9">
+        <f>$M2*(1-Calculations!Q3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="R3" s="9">
-        <f>$M3*(1-Calculations!R3)</f>
+      <c r="R2" s="9">
+        <f>$M2*(1-Calculations!R3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="S3" s="9">
-        <f>$M3*(1-Calculations!S3)</f>
+      <c r="S2" s="9">
+        <f>$M2*(1-Calculations!S3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="T3" s="9">
-        <f>$M3*(1-Calculations!T3)</f>
+      <c r="T2" s="9">
+        <f>$M2*(1-Calculations!T3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="U3" s="9">
-        <f>$M3*(1-Calculations!U3)</f>
+      <c r="U2" s="9">
+        <f>$M2*(1-Calculations!U3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="V3" s="9">
-        <f>$M3*(1-Calculations!V3)</f>
+      <c r="V2" s="9">
+        <f>$M2*(1-Calculations!V3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="W3" s="9">
-        <f>$M3*(1-Calculations!W3)</f>
+      <c r="W2" s="9">
+        <f>$M2*(1-Calculations!W3)</f>
         <v>60.65753899562943</v>
       </c>
-      <c r="X3" s="9">
-        <f>$M3*(1-Calculations!X3)</f>
+      <c r="X2" s="9">
+        <f>$M2*(1-Calculations!X3)</f>
         <v>48.526031196503546</v>
       </c>
-      <c r="Y3" s="9">
-        <f>$M3*(1-Calculations!Y3)</f>
+      <c r="Y2" s="9">
+        <f>$M2*(1-Calculations!Y3)</f>
         <v>36.394523397377654</v>
       </c>
-      <c r="Z3" s="9">
-        <f>$M3*(1-Calculations!Z3)</f>
+      <c r="Z2" s="9">
+        <f>$M2*(1-Calculations!Z3)</f>
         <v>24.263015598251766</v>
       </c>
-      <c r="AA3" s="9">
-        <f>$M3*(1-Calculations!AA3)</f>
+      <c r="AA2" s="9">
+        <f>$M2*(1-Calculations!AA3)</f>
         <v>12.131507799125883</v>
       </c>
-      <c r="AB3" s="9">
-        <f>$M3*(1-Calculations!AB3)</f>
-        <v>0</v>
-      </c>
-      <c r="AC3" s="9">
-        <f>$M3*(1-Calculations!AC3)</f>
-        <v>0</v>
-      </c>
-      <c r="AD3" s="9">
-        <f>$M3*(1-Calculations!AD3)</f>
-        <v>0</v>
-      </c>
-      <c r="AE3" s="9">
-        <f>$M3*(1-Calculations!AE3)</f>
+      <c r="AB2" s="9">
+        <f>$M2*(1-Calculations!AB3)</f>
+        <v>0</v>
+      </c>
+      <c r="AC2" s="9">
+        <f>$M2*(1-Calculations!AC3)</f>
+        <v>0</v>
+      </c>
+      <c r="AD2" s="9">
+        <f>$M2*(1-Calculations!AD3)</f>
+        <v>0</v>
+      </c>
+      <c r="AE2" s="9">
+        <f>$M2*(1-Calculations!AE3)</f>
         <v>0</v>
       </c>
     </row>
@@ -2198,6 +2172,2499 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F89E83AC-E3AB-43F2-AEFA-7AD478FA75F7}">
+  <sheetPr>
+    <tabColor theme="3"/>
+  </sheetPr>
+  <dimension ref="A1:AE25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1">
+        <v>2021</v>
+      </c>
+      <c r="C1">
+        <v>2022</v>
+      </c>
+      <c r="D1">
+        <v>2023</v>
+      </c>
+      <c r="E1">
+        <v>2024</v>
+      </c>
+      <c r="F1">
+        <v>2025</v>
+      </c>
+      <c r="G1">
+        <v>2026</v>
+      </c>
+      <c r="H1">
+        <v>2027</v>
+      </c>
+      <c r="I1">
+        <v>2028</v>
+      </c>
+      <c r="J1">
+        <v>2029</v>
+      </c>
+      <c r="K1">
+        <v>2030</v>
+      </c>
+      <c r="L1">
+        <v>2031</v>
+      </c>
+      <c r="M1">
+        <v>2032</v>
+      </c>
+      <c r="N1">
+        <v>2033</v>
+      </c>
+      <c r="O1">
+        <v>2034</v>
+      </c>
+      <c r="P1">
+        <v>2035</v>
+      </c>
+      <c r="Q1">
+        <v>2036</v>
+      </c>
+      <c r="R1">
+        <v>2037</v>
+      </c>
+      <c r="S1">
+        <v>2038</v>
+      </c>
+      <c r="T1">
+        <v>2039</v>
+      </c>
+      <c r="U1">
+        <v>2040</v>
+      </c>
+      <c r="V1">
+        <v>2041</v>
+      </c>
+      <c r="W1">
+        <v>2042</v>
+      </c>
+      <c r="X1">
+        <v>2043</v>
+      </c>
+      <c r="Y1">
+        <v>2044</v>
+      </c>
+      <c r="Z1">
+        <v>2045</v>
+      </c>
+      <c r="AA1">
+        <v>2046</v>
+      </c>
+      <c r="AB1">
+        <v>2047</v>
+      </c>
+      <c r="AC1">
+        <v>2048</v>
+      </c>
+      <c r="AD1">
+        <v>2049</v>
+      </c>
+      <c r="AE1">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>0</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
+        <v>0</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
+      <c r="AE6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>0</v>
+      </c>
+      <c r="AB7">
+        <v>0</v>
+      </c>
+      <c r="AC7">
+        <v>0</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+      <c r="AE7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>0</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>0</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+      <c r="AE8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
+        <v>0</v>
+      </c>
+      <c r="AB9">
+        <v>0</v>
+      </c>
+      <c r="AC9">
+        <v>0</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+      <c r="AE9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
+      </c>
+      <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>98</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>0</v>
+      </c>
+      <c r="Y12">
+        <v>0</v>
+      </c>
+      <c r="Z12">
+        <v>0</v>
+      </c>
+      <c r="AA12">
+        <v>0</v>
+      </c>
+      <c r="AB12">
+        <v>0</v>
+      </c>
+      <c r="AC12">
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <v>0</v>
+      </c>
+      <c r="AE12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>0</v>
+      </c>
+      <c r="Y13">
+        <v>0</v>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
+        <v>0</v>
+      </c>
+      <c r="AB13">
+        <v>0</v>
+      </c>
+      <c r="AC13">
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+      <c r="AE13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>0</v>
+      </c>
+      <c r="AB14">
+        <v>0</v>
+      </c>
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>0</v>
+      </c>
+      <c r="AB15">
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+      <c r="AE15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <v>0</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>0</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+      <c r="AA16">
+        <v>0</v>
+      </c>
+      <c r="AB16">
+        <v>0</v>
+      </c>
+      <c r="AC16">
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <v>0</v>
+      </c>
+      <c r="AE16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <v>0</v>
+      </c>
+      <c r="Z17">
+        <v>0</v>
+      </c>
+      <c r="AA17">
+        <v>0</v>
+      </c>
+      <c r="AB17">
+        <v>0</v>
+      </c>
+      <c r="AC17">
+        <v>0</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+      <c r="AE17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>0</v>
+      </c>
+      <c r="Y18">
+        <v>0</v>
+      </c>
+      <c r="Z18">
+        <v>0</v>
+      </c>
+      <c r="AA18">
+        <v>0</v>
+      </c>
+      <c r="AB18">
+        <v>0</v>
+      </c>
+      <c r="AC18">
+        <v>0</v>
+      </c>
+      <c r="AD18">
+        <v>0</v>
+      </c>
+      <c r="AE18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="9">
+        <f>'BCS-industry'!B2</f>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C19" s="9">
+        <f>'BCS-industry'!C2</f>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D19" s="9">
+        <f>'BCS-industry'!D2</f>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E19" s="9">
+        <f>'BCS-industry'!E2</f>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F19" s="9">
+        <f>'BCS-industry'!F2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G19" s="9">
+        <f>'BCS-industry'!G2</f>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H19" s="9">
+        <f>'BCS-industry'!H2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I19" s="9">
+        <f>'BCS-industry'!I2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J19" s="9">
+        <f>'BCS-industry'!J2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K19" s="9">
+        <f>'BCS-industry'!K2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L19" s="9">
+        <f>'BCS-industry'!L2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M19" s="9">
+        <f>'BCS-industry'!M2</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <v>0</v>
+      </c>
+      <c r="V19">
+        <v>0</v>
+      </c>
+      <c r="W19">
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <v>0</v>
+      </c>
+      <c r="Y19">
+        <v>0</v>
+      </c>
+      <c r="Z19">
+        <v>0</v>
+      </c>
+      <c r="AA19">
+        <v>0</v>
+      </c>
+      <c r="AB19">
+        <v>0</v>
+      </c>
+      <c r="AC19">
+        <v>0</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
+      </c>
+      <c r="AE19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="11">
+        <f>B19</f>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C20" s="11">
+        <f t="shared" ref="C20:C22" si="0">C19</f>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D20" s="11">
+        <f t="shared" ref="D20:D22" si="1">D19</f>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E20" s="11">
+        <f t="shared" ref="E20:E22" si="2">E19</f>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F20" s="11">
+        <f t="shared" ref="F20:F22" si="3">F19</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G20" s="11">
+        <f t="shared" ref="G20:G22" si="4">G19</f>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H20" s="11">
+        <f t="shared" ref="H20:H22" si="5">H19</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I20" s="11">
+        <f t="shared" ref="I20:I22" si="6">I19</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J20" s="11">
+        <f t="shared" ref="J20:J22" si="7">J19</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K20" s="11">
+        <f t="shared" ref="K20:K22" si="8">K19</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L20" s="11">
+        <f t="shared" ref="L20:L22" si="9">L19</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M20" s="11">
+        <f t="shared" ref="M20:M22" si="10">M19</f>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N20" s="11">
+        <f t="shared" ref="N20:N22" si="11">N19</f>
+        <v>0</v>
+      </c>
+      <c r="O20" s="11">
+        <f t="shared" ref="O20:O22" si="12">O19</f>
+        <v>0</v>
+      </c>
+      <c r="P20" s="11">
+        <f t="shared" ref="P20:P22" si="13">P19</f>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="11">
+        <f t="shared" ref="Q20:Q22" si="14">Q19</f>
+        <v>0</v>
+      </c>
+      <c r="R20" s="11">
+        <f t="shared" ref="R20:R22" si="15">R19</f>
+        <v>0</v>
+      </c>
+      <c r="S20" s="11">
+        <f t="shared" ref="S20:S22" si="16">S19</f>
+        <v>0</v>
+      </c>
+      <c r="T20" s="11">
+        <f t="shared" ref="T20:T22" si="17">T19</f>
+        <v>0</v>
+      </c>
+      <c r="U20" s="11">
+        <f t="shared" ref="U20:U22" si="18">U19</f>
+        <v>0</v>
+      </c>
+      <c r="V20" s="11">
+        <f t="shared" ref="V20:V22" si="19">V19</f>
+        <v>0</v>
+      </c>
+      <c r="W20" s="11">
+        <f t="shared" ref="W20:W22" si="20">W19</f>
+        <v>0</v>
+      </c>
+      <c r="X20" s="11">
+        <f t="shared" ref="X20:X22" si="21">X19</f>
+        <v>0</v>
+      </c>
+      <c r="Y20" s="11">
+        <f t="shared" ref="Y20:Y22" si="22">Y19</f>
+        <v>0</v>
+      </c>
+      <c r="Z20" s="11">
+        <f t="shared" ref="Z20:Z22" si="23">Z19</f>
+        <v>0</v>
+      </c>
+      <c r="AA20" s="11">
+        <f t="shared" ref="AA20:AA22" si="24">AA19</f>
+        <v>0</v>
+      </c>
+      <c r="AB20" s="11">
+        <f t="shared" ref="AB20:AB22" si="25">AB19</f>
+        <v>0</v>
+      </c>
+      <c r="AC20" s="11">
+        <f t="shared" ref="AC20:AC22" si="26">AC19</f>
+        <v>0</v>
+      </c>
+      <c r="AD20" s="11">
+        <f t="shared" ref="AD20:AD22" si="27">AD19</f>
+        <v>0</v>
+      </c>
+      <c r="AE20" s="11">
+        <f t="shared" ref="AE20:AE22" si="28">AE19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" s="11">
+        <f t="shared" ref="B21:B22" si="29">B20</f>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C21" s="11">
+        <f t="shared" si="0"/>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D21" s="11">
+        <f t="shared" si="1"/>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E21" s="11">
+        <f t="shared" si="2"/>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F21" s="11">
+        <f t="shared" si="3"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G21" s="11">
+        <f t="shared" si="4"/>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H21" s="11">
+        <f t="shared" si="5"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I21" s="11">
+        <f t="shared" si="6"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J21" s="11">
+        <f t="shared" si="7"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K21" s="11">
+        <f t="shared" si="8"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L21" s="11">
+        <f t="shared" si="9"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M21" s="11">
+        <f t="shared" si="10"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N21" s="11">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O21" s="11">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="P21" s="11">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="Q21" s="11">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="R21" s="11">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="S21" s="11">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="T21" s="11">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="U21" s="11">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="V21" s="11">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="W21" s="11">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X21" s="11">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="Y21" s="11">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="Z21" s="11">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="AA21" s="11">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="AB21" s="11">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
+      <c r="AC21" s="11">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="AD21" s="11">
+        <f t="shared" si="27"/>
+        <v>0</v>
+      </c>
+      <c r="AE21" s="11">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="11">
+        <f t="shared" si="29"/>
+        <v>42.365206480422181</v>
+      </c>
+      <c r="C22" s="11">
+        <f t="shared" si="0"/>
+        <v>39.226051152380791</v>
+      </c>
+      <c r="D22" s="11">
+        <f t="shared" si="1"/>
+        <v>64.04779095640987</v>
+      </c>
+      <c r="E22" s="11">
+        <f t="shared" si="2"/>
+        <v>62.212860508337869</v>
+      </c>
+      <c r="F22" s="11">
+        <f t="shared" si="3"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="G22" s="11">
+        <f t="shared" si="4"/>
+        <v>59.141100520738689</v>
+      </c>
+      <c r="H22" s="11">
+        <f t="shared" si="5"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="I22" s="11">
+        <f t="shared" si="6"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="J22" s="11">
+        <f t="shared" si="7"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="K22" s="11">
+        <f t="shared" si="8"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="L22" s="11">
+        <f t="shared" si="9"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="M22" s="11">
+        <f t="shared" si="10"/>
+        <v>60.65753899562943</v>
+      </c>
+      <c r="N22" s="11">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="O22" s="11">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="P22" s="11">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="11">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="R22" s="11">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="S22" s="11">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="T22" s="11">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="U22" s="11">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="V22" s="11">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="W22" s="11">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X22" s="11">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="Y22" s="11">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="Z22" s="11">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="AA22" s="11">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="AB22" s="11">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
+      <c r="AC22" s="11">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="AD22" s="11">
+        <f t="shared" si="27"/>
+        <v>0</v>
+      </c>
+      <c r="AE22" s="11">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>0</v>
+      </c>
+      <c r="U23">
+        <v>0</v>
+      </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="Y23">
+        <v>0</v>
+      </c>
+      <c r="Z23">
+        <v>0</v>
+      </c>
+      <c r="AA23">
+        <v>0</v>
+      </c>
+      <c r="AB23">
+        <v>0</v>
+      </c>
+      <c r="AC23">
+        <v>0</v>
+      </c>
+      <c r="AD23">
+        <v>0</v>
+      </c>
+      <c r="AE23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>0</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <v>0</v>
+      </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+      <c r="W24">
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
+      <c r="Y24">
+        <v>0</v>
+      </c>
+      <c r="Z24">
+        <v>0</v>
+      </c>
+      <c r="AA24">
+        <v>0</v>
+      </c>
+      <c r="AB24">
+        <v>0</v>
+      </c>
+      <c r="AC24">
+        <v>0</v>
+      </c>
+      <c r="AD24">
+        <v>0</v>
+      </c>
+      <c r="AE24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>0</v>
+      </c>
+      <c r="U25">
+        <v>0</v>
+      </c>
+      <c r="V25">
+        <v>0</v>
+      </c>
+      <c r="W25">
+        <v>0</v>
+      </c>
+      <c r="X25">
+        <v>0</v>
+      </c>
+      <c r="Y25">
+        <v>0</v>
+      </c>
+      <c r="Z25">
+        <v>0</v>
+      </c>
+      <c r="AA25">
+        <v>0</v>
+      </c>
+      <c r="AB25">
+        <v>0</v>
+      </c>
+      <c r="AC25">
+        <v>0</v>
+      </c>
+      <c r="AD25">
+        <v>0</v>
+      </c>
+      <c r="AE25">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5698252-CD29-4D86-9D7F-2214C5598602}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -2207,7 +4674,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1">
         <v>2021</v>
@@ -2302,7 +4769,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2">
         <v>12</v>

</xml_diff>

<commit_message>
Correct currency year for 45Q tax credits
</commit_message>
<xml_diff>
--- a/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
+++ b/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ccs\BCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7519D7CE-E98F-413E-A6DF-5C9601EE62D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278F3552-43BC-45DE-9C0A-8ADFD495AF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -55,6 +55,9 @@
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -109,12 +112,6 @@
     <t>https://www.bls.gov/data/inflation_calculator.htm</t>
   </si>
   <si>
-    <t>2024 to 2012 USD</t>
-  </si>
-  <si>
-    <t>*inflation adjusted starting in 2025, so we use the 2024 currency year to adjust to 2012 $</t>
-  </si>
-  <si>
     <t>45Q tax credits include a commenced construction provision. Based on EIA data, we assume a construction timeline</t>
   </si>
   <si>
@@ -230,6 +227,12 @@
   </si>
   <si>
     <t>values for industry only to reflect the duration multiplier.</t>
+  </si>
+  <si>
+    <t>2025 to 2012 USD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*26 U.S.C. 45Q(h): inflation adjustment applies to taxable years beginning after 2026, substituting 2025 for 1990 - so the $85 is in 2025 dollars and we use the 2025 currency year to adjust to 2012 $. Factor matches the model OCCF (0.713109). </t>
   </si>
 </sst>
 </file>
@@ -664,19 +667,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C56"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.81640625" customWidth="1"/>
-    <col min="2" max="2" width="55.81640625" customWidth="1"/>
-    <col min="4" max="4" width="30.54296875" customWidth="1"/>
+    <col min="1" max="1" width="41.85546875" customWidth="1"/>
+    <col min="2" max="2" width="55.85546875" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -684,33 +687,33 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
-        <v>0.73</v>
+        <v>0.71310899999999999</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
@@ -718,13 +721,13 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="B12" s="5"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -732,29 +735,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -767,12 +770,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1086F14D-0ABA-4CBC-A6C8-8AA6F7BA1ED0}">
   <dimension ref="A1:AE35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B1" s="6">
         <v>2021</v>
       </c>
@@ -864,9 +867,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -964,9 +967,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <f>IFERROR(IF(A3=1,1,INDEX($B$2:$AE$2,MATCH((B1-'BCS-DoSfCS'!$B$2),$B$1:$AE$1,0))),0)</f>
@@ -1089,22 +1092,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>2022</v>
       </c>
@@ -1115,19 +1118,19 @@
         <v>2035</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>24</v>
       </c>
       <c r="B12">
         <v>14</v>
@@ -1139,34 +1142,34 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>30</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1178,12 +1181,12 @@
         <v>60</v>
       </c>
       <c r="E18" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B19">
         <v>2</v>
@@ -1195,30 +1198,30 @@
         <v>53</v>
       </c>
       <c r="E19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>34</v>
       </c>
-      <c r="E20" t="s">
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>38</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -1230,9 +1233,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -1244,59 +1247,59 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1310,13 +1313,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.453125" customWidth="1"/>
-    <col min="2" max="2" width="24.54296875" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -1411,7 +1414,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1423,55 +1426,55 @@
       </c>
       <c r="D2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="E2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="F2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="G2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="H2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="I2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="J2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="K2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="L2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="M2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="N2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="O2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="P2">
         <f>About!$B$11*About!$A$9</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -1519,7 +1522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1531,99 +1534,99 @@
       </c>
       <c r="D3">
         <f>About!$B$11*About!$A$9*(1-Calculations!D3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="E3">
         <f>About!$B$11*About!$A$9*(1-Calculations!E3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="F3">
         <f>About!$B$11*About!$A$9*(1-Calculations!F3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="G3">
         <f>About!$B$11*About!$A$9*(1-Calculations!G3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="H3">
         <f>About!$B$11*About!$A$9*(1-Calculations!H3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="I3">
         <f>About!$B$11*About!$A$9*(1-Calculations!I3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="J3">
         <f>About!$B$11*About!$A$9*(1-Calculations!J3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="K3">
         <f>About!$B$11*About!$A$9*(1-Calculations!K3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="L3">
         <f>About!$B$11*About!$A$9*(1-Calculations!L3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="M3">
         <f>About!$B$11*About!$A$9*(1-Calculations!M3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="N3">
         <f>About!$B$11*About!$A$9*(1-Calculations!N3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="O3">
         <f>About!$B$11*About!$A$9*(1-Calculations!O3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="P3">
         <f>About!$B$11*About!$A$9*(1-Calculations!P3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="Q3">
         <f>About!$B$11*About!$A$9*(1-Calculations!Q3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="R3">
         <f>About!$B$11*About!$A$9*(1-Calculations!R3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="S3">
         <f>About!$B$11*About!$A$9*(1-Calculations!S3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="T3">
         <f>About!$B$11*About!$A$9*(1-Calculations!T3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="U3">
         <f>About!$B$11*About!$A$9*(1-Calculations!U3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="V3">
         <f>About!$B$11*About!$A$9*(1-Calculations!V3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="W3">
         <f>About!$B$11*About!$A$9*(1-Calculations!W3)</f>
-        <v>62.05</v>
+        <v>60.614264999999996</v>
       </c>
       <c r="X3">
         <f>About!$B$11*About!$A$9*(1-Calculations!X3)</f>
-        <v>49.64</v>
+        <v>48.491411999999997</v>
       </c>
       <c r="Y3">
         <f>About!$B$11*About!$A$9*(1-Calculations!Y3)</f>
-        <v>37.229999999999997</v>
+        <v>36.368558999999998</v>
       </c>
       <c r="Z3">
         <f>About!$B$11*About!$A$9*(1-Calculations!Z3)</f>
-        <v>24.819999999999993</v>
+        <v>24.245705999999991</v>
       </c>
       <c r="AA3">
         <f>About!$B$11*About!$A$9*(1-Calculations!AA3)</f>
-        <v>12.409999999999997</v>
+        <v>12.122852999999996</v>
       </c>
       <c r="AB3">
         <f>About!$B$11*About!$A$9*(1-Calculations!AB3)</f>
@@ -1653,9 +1656,9 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -1750,7 +1753,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>

</xml_diff>